<commit_message>
fix(ukelonn): close source workflow parity gaps
</commit_message>
<xml_diff>
--- a/tests/fixtures/ukelonn-import-synthetic.xlsx
+++ b/tests/fixtures/ukelonn-import-synthetic.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Demo" sheetId="1" r:id="rId1"/>
+    <sheet name="Gjøremål" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -23,6 +23,11 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Aktiv</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Bilde kreves</t>
         </is>
       </c>
@@ -38,7 +43,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Syntetisk inaktiv oppgave</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>5.00</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ja</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ukelonn): close source workflow parity gaps (#98)
Co-authored-by: Eirik Yven <eirik@yven.me>
</commit_message>
<xml_diff>
--- a/tests/fixtures/ukelonn-import-synthetic.xlsx
+++ b/tests/fixtures/ukelonn-import-synthetic.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Demo" sheetId="1" r:id="rId1"/>
+    <sheet name="Gjøremål" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -23,6 +23,11 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Aktiv</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Bilde kreves</t>
         </is>
       </c>
@@ -38,7 +43,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Syntetisk inaktiv oppgave</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>5.00</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ja</t>
         </is>
       </c>
     </row>

</xml_diff>